<commit_message>
TableManager 수정 및 ClientLocalStorage 리펙토링 진행
</commit_message>
<xml_diff>
--- a/DesignTable/Data/Table/Tables/AtlasData.xlsx
+++ b/DesignTable/Data/Table/Tables/AtlasData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\ProjectT\DesignTable\Data\Table\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79CDA281-AFE3-4CF5-AFB9-8D44CA9A5869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD976AF5-E506-4EEB-83DE-ED2FA22BD1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3F4DC61C-DF7F-4950-B9C6-A6313E9C3BA7}"/>
   </bookViews>
@@ -213,7 +213,7 @@
       </xsd:element>
     </xsd:schema>
   </Schema>
-  <Map ID="7" Name="AtlasData_맵" RootElement="AtlasData" SchemaID="Schema2" ShowImportExportValidationErrors="false" AutoFit="true" Append="false" PreserveSortAFLayout="true" PreserveFormat="true"/>
+  <Map ID="9" Name="AtlasData_맵" RootElement="AtlasData" SchemaID="Schema2" ShowImportExportValidationErrors="false" AutoFit="true" Append="false" PreserveSortAFLayout="true" PreserveFormat="true"/>
 </MapInfo>
 </file>
 
@@ -222,10 +222,10 @@
   <autoFilter ref="A1:B2" xr:uid="{13BD990D-B10A-4799-B394-70076236F817}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{3E14796D-9F90-41FD-8685-10B2F06916CA}" uniqueName="AtlasType" name="AtlasType">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/record/AtlasType" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/record/AtlasType" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{742E6A75-7DEA-4AAE-B8CF-CB3FCCBBFB7B}" uniqueName="Path" name="Path">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/record/Path" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/record/Path" xmlDataType="string"/>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -237,34 +237,34 @@
   <autoFilter ref="A1:J3" xr:uid="{7B4B12F9-7C42-4143-8B3D-BFDB82DEDFC3}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9AC35F50-B3BB-4A8A-81B2-1722DCB2A5CE}" uniqueName="ColumnName" name="ColumnName">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/verify/@ColumnName" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@ColumnName" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{EB278A5B-ED8E-4AA2-BD5E-B1CE80E221FF}" uniqueName="Type" name="Type">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/verify/@Type" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@Type" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{CC864C3D-D82D-4B7D-805A-41EB891F0133}" uniqueName="IsClient" name="IsClient">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/verify/@IsClient" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@IsClient" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{7EF56112-C93B-49FB-A525-847DB5DF9C2E}" uniqueName="IsServer" name="IsServer">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/verify/@IsServer" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@IsServer" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{7BC6B606-3953-4A21-B87D-B1617FAF3191}" uniqueName="PK" name="PK">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/verify/@PK" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@PK" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{D04FB710-3E13-48FC-BBB9-1D63CE687FA1}" uniqueName="EnumID" name="EnumID">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/verify/@EnumID" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@EnumID" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{CD2A9EDE-3E08-43D3-A0E8-75327CB4BA61}" uniqueName="IDRule" name="IDRule">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/verify/@IDRule" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@IDRule" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{7FB2C5DD-4B14-49C8-AA33-FAEDB62D5E59}" uniqueName="StringHashIds" name="StringHashIds">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/verify/@StringHashIds" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@StringHashIds" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="9" xr3:uid="{5A8A3B69-FC59-43C8-8C40-8CA28ACF7E75}" uniqueName="FieldNo" name="FieldNo">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/verify/@FieldNo" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@FieldNo" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{0CE418AC-4A34-4DC2-91D8-E190D96A4DC7}" uniqueName="TableId" name="TableId" dataDxfId="0">
-      <xmlColumnPr mapId="7" xpath="/AtlasData/verify/@TableId" xmlDataType="string"/>
+      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@TableId" xmlDataType="string"/>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>

</xml_diff>

<commit_message>
Notify, Sound, Controller 시스템 리펙토링
</commit_message>
<xml_diff>
--- a/DesignTable/Data/Table/Tables/AtlasData.xlsx
+++ b/DesignTable/Data/Table/Tables/AtlasData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\ProjectT\DesignTable\Data\Table\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD976AF5-E506-4EEB-83DE-ED2FA22BD1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{555D1677-ABA9-482D-AC8A-20BC20798247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3F4DC61C-DF7F-4950-B9C6-A6313E9C3BA7}"/>
   </bookViews>
@@ -213,7 +213,7 @@
       </xsd:element>
     </xsd:schema>
   </Schema>
-  <Map ID="9" Name="AtlasData_맵" RootElement="AtlasData" SchemaID="Schema2" ShowImportExportValidationErrors="false" AutoFit="true" Append="false" PreserveSortAFLayout="true" PreserveFormat="true"/>
+  <Map ID="10" Name="AtlasData_맵" RootElement="AtlasData" SchemaID="Schema2" ShowImportExportValidationErrors="false" AutoFit="true" Append="false" PreserveSortAFLayout="true" PreserveFormat="true"/>
 </MapInfo>
 </file>
 
@@ -222,10 +222,10 @@
   <autoFilter ref="A1:B2" xr:uid="{13BD990D-B10A-4799-B394-70076236F817}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{3E14796D-9F90-41FD-8685-10B2F06916CA}" uniqueName="AtlasType" name="AtlasType">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/record/AtlasType" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/record/AtlasType" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{742E6A75-7DEA-4AAE-B8CF-CB3FCCBBFB7B}" uniqueName="Path" name="Path">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/record/Path" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/record/Path" xmlDataType="string"/>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -237,34 +237,34 @@
   <autoFilter ref="A1:J3" xr:uid="{7B4B12F9-7C42-4143-8B3D-BFDB82DEDFC3}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9AC35F50-B3BB-4A8A-81B2-1722DCB2A5CE}" uniqueName="ColumnName" name="ColumnName">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@ColumnName" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/verify/@ColumnName" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{EB278A5B-ED8E-4AA2-BD5E-B1CE80E221FF}" uniqueName="Type" name="Type">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@Type" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/verify/@Type" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{CC864C3D-D82D-4B7D-805A-41EB891F0133}" uniqueName="IsClient" name="IsClient">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@IsClient" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/verify/@IsClient" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{7EF56112-C93B-49FB-A525-847DB5DF9C2E}" uniqueName="IsServer" name="IsServer">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@IsServer" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/verify/@IsServer" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{7BC6B606-3953-4A21-B87D-B1617FAF3191}" uniqueName="PK" name="PK">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@PK" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/verify/@PK" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{D04FB710-3E13-48FC-BBB9-1D63CE687FA1}" uniqueName="EnumID" name="EnumID">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@EnumID" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/verify/@EnumID" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{CD2A9EDE-3E08-43D3-A0E8-75327CB4BA61}" uniqueName="IDRule" name="IDRule">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@IDRule" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/verify/@IDRule" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{7FB2C5DD-4B14-49C8-AA33-FAEDB62D5E59}" uniqueName="StringHashIds" name="StringHashIds">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@StringHashIds" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/verify/@StringHashIds" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="9" xr3:uid="{5A8A3B69-FC59-43C8-8C40-8CA28ACF7E75}" uniqueName="FieldNo" name="FieldNo">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@FieldNo" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/verify/@FieldNo" xmlDataType="string"/>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{0CE418AC-4A34-4DC2-91D8-E190D96A4DC7}" uniqueName="TableId" name="TableId" dataDxfId="0">
-      <xmlColumnPr mapId="9" xpath="/AtlasData/verify/@TableId" xmlDataType="string"/>
+      <xmlColumnPr mapId="10" xpath="/AtlasData/verify/@TableId" xmlDataType="string"/>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>

</xml_diff>